<commit_message>
Add the third annotation batch (95 EP sentences) and harden the loaders
Convert the Abergaria workbook with the existing ingest script: its own
column layout and tense spellings are mapped (judgement calls documented),
three duplicates are dropped and reported, IDs are PTEUJ1..95. Sentence
grouping for CV now ignores digits, punctuation and quotes so near-duplicates
(PTAO36 / PTAOV25) share a fold. Blank SR-SC/DR are accepted only in the
later batches, load(path=...) no longer treats an empty path as "no path",
sheets are resolved through the workbook relationships, and personal
metadata is scrubbed from the committed Violeta workbook.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/archive/Dados_Violeta.xlsx
+++ b/data/raw/archive/Dados_Violeta.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Puri/Desktop/DRIPPS/"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{F62DFBE9-5699-6546-81A8-3253B9BE0735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>